<commit_message>
(feature) [AC-383] : Student Spoken Language and Proficiency
</commit_message>
<xml_diff>
--- a/database/ddml-new/ServiceSubjects.xlsx
+++ b/database/ddml-new/ServiceSubjects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kimoy\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SourceCloud\academically-app\database\ddml-new\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0B13BC-B5B9-487B-ABDB-926016ADC241}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00001BC7-13EA-49C0-925F-82D7432ABFC8}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{43392282-EF0F-4456-BB12-6FFFCECE476B}"/>
   </bookViews>
@@ -42,9 +42,6 @@
     <t>SubjectId</t>
   </si>
   <si>
-    <t>f4c0dbdb-1144-431e-ae0f-f52fa4867703</t>
-  </si>
-  <si>
     <t>74762a44-1264-44e3-a471-d98b3facf1cb</t>
   </si>
   <si>
@@ -318,7 +315,10 @@
     <t>4b876da1-2d6e-4c19-b01b-e7a8e9ca67bb</t>
   </si>
   <si>
-    <t>b060591f-e4a8-4552-9903-0fbf41c6ed66</t>
+    <t>6aa0d3b8-6229-4945-809a-a704f39b1b22</t>
+  </si>
+  <si>
+    <t>9a8d9777-ead3-4344-af27-d9a595f5de5c</t>
   </si>
 </sst>
 </file>
@@ -694,130 +694,130 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -825,7 +825,7 @@
         <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -833,7 +833,7 @@
         <v>94</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -841,7 +841,7 @@
         <v>94</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -849,7 +849,7 @@
         <v>94</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -857,7 +857,7 @@
         <v>94</v>
       </c>
       <c r="B22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -865,7 +865,7 @@
         <v>94</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -873,7 +873,7 @@
         <v>94</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -881,7 +881,7 @@
         <v>94</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -889,7 +889,7 @@
         <v>94</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -897,7 +897,7 @@
         <v>94</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -905,7 +905,7 @@
         <v>94</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -913,7 +913,7 @@
         <v>94</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -921,7 +921,7 @@
         <v>94</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -929,7 +929,7 @@
         <v>94</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -937,7 +937,7 @@
         <v>94</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -945,7 +945,7 @@
         <v>94</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -953,7 +953,7 @@
         <v>94</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -961,7 +961,7 @@
         <v>94</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -969,7 +969,7 @@
         <v>94</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -977,7 +977,7 @@
         <v>94</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -985,7 +985,7 @@
         <v>94</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -993,7 +993,7 @@
         <v>94</v>
       </c>
       <c r="B39" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -1001,7 +1001,7 @@
         <v>94</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -1009,7 +1009,7 @@
         <v>94</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -1017,7 +1017,7 @@
         <v>94</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -1025,7 +1025,7 @@
         <v>94</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -1033,7 +1033,7 @@
         <v>94</v>
       </c>
       <c r="B44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -1041,7 +1041,7 @@
         <v>94</v>
       </c>
       <c r="B45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -1049,7 +1049,7 @@
         <v>94</v>
       </c>
       <c r="B46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -1057,7 +1057,7 @@
         <v>94</v>
       </c>
       <c r="B47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -1065,7 +1065,7 @@
         <v>94</v>
       </c>
       <c r="B48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -1073,7 +1073,7 @@
         <v>94</v>
       </c>
       <c r="B49" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -1081,7 +1081,7 @@
         <v>94</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -1089,7 +1089,7 @@
         <v>94</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -1097,7 +1097,7 @@
         <v>94</v>
       </c>
       <c r="B52" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -1105,7 +1105,7 @@
         <v>94</v>
       </c>
       <c r="B53" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -1113,7 +1113,7 @@
         <v>94</v>
       </c>
       <c r="B54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -1121,7 +1121,7 @@
         <v>94</v>
       </c>
       <c r="B55" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>94</v>
       </c>
       <c r="B56" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -1137,7 +1137,7 @@
         <v>94</v>
       </c>
       <c r="B57" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -1145,7 +1145,7 @@
         <v>94</v>
       </c>
       <c r="B58" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -1153,7 +1153,7 @@
         <v>94</v>
       </c>
       <c r="B59" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -1161,7 +1161,7 @@
         <v>94</v>
       </c>
       <c r="B60" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -1169,7 +1169,7 @@
         <v>94</v>
       </c>
       <c r="B61" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -1177,7 +1177,7 @@
         <v>94</v>
       </c>
       <c r="B62" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -1185,7 +1185,7 @@
         <v>94</v>
       </c>
       <c r="B63" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -1193,7 +1193,7 @@
         <v>94</v>
       </c>
       <c r="B64" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -1201,7 +1201,7 @@
         <v>94</v>
       </c>
       <c r="B65" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -1209,7 +1209,7 @@
         <v>94</v>
       </c>
       <c r="B66" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -1217,7 +1217,7 @@
         <v>94</v>
       </c>
       <c r="B67" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -1225,7 +1225,7 @@
         <v>94</v>
       </c>
       <c r="B68" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>94</v>
       </c>
       <c r="B69" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -1241,7 +1241,7 @@
         <v>94</v>
       </c>
       <c r="B70" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -1249,7 +1249,7 @@
         <v>94</v>
       </c>
       <c r="B71" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -1257,7 +1257,7 @@
         <v>94</v>
       </c>
       <c r="B72" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -1265,7 +1265,7 @@
         <v>94</v>
       </c>
       <c r="B73" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -1273,7 +1273,7 @@
         <v>94</v>
       </c>
       <c r="B74" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -1281,7 +1281,7 @@
         <v>94</v>
       </c>
       <c r="B75" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -1289,7 +1289,7 @@
         <v>94</v>
       </c>
       <c r="B76" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -1297,7 +1297,7 @@
         <v>94</v>
       </c>
       <c r="B77" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -1305,7 +1305,7 @@
         <v>94</v>
       </c>
       <c r="B78" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -1313,7 +1313,7 @@
         <v>94</v>
       </c>
       <c r="B79" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
@@ -1321,7 +1321,7 @@
         <v>94</v>
       </c>
       <c r="B80" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
@@ -1329,7 +1329,7 @@
         <v>94</v>
       </c>
       <c r="B81" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
@@ -1337,7 +1337,7 @@
         <v>94</v>
       </c>
       <c r="B82" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
@@ -1345,7 +1345,7 @@
         <v>94</v>
       </c>
       <c r="B83" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -1353,7 +1353,7 @@
         <v>94</v>
       </c>
       <c r="B84" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -1361,7 +1361,7 @@
         <v>94</v>
       </c>
       <c r="B85" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
@@ -1369,7 +1369,7 @@
         <v>94</v>
       </c>
       <c r="B86" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
@@ -1377,7 +1377,7 @@
         <v>94</v>
       </c>
       <c r="B87" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
@@ -1385,7 +1385,7 @@
         <v>94</v>
       </c>
       <c r="B88" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
@@ -1393,7 +1393,7 @@
         <v>94</v>
       </c>
       <c r="B89" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
@@ -1401,7 +1401,7 @@
         <v>94</v>
       </c>
       <c r="B90" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -1409,7 +1409,7 @@
         <v>94</v>
       </c>
       <c r="B91" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -1417,7 +1417,7 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -1425,7 +1425,7 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -1433,7 +1433,7 @@
         <v>94</v>
       </c>
       <c r="B94" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
@@ -1441,7 +1441,7 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
@@ -1449,7 +1449,7 @@
         <v>94</v>
       </c>
       <c r="B96" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
@@ -1457,7 +1457,7 @@
         <v>94</v>
       </c>
       <c r="B97" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>